<commit_message>
fix: reach exactly 100 products in day-0 import template when data supports it
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/seed_data/day0_import_template.sample.xlsx
+++ b/backend/seed_data/day0_import_template.sample.xlsx
@@ -451,376 +451,376 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Frozen Peas 500g</t>
+          <t>Chicken Breast 1kg</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SKU-DEMO-FROZEN-001</t>
+          <t>SKU-DEMO-MEAT-001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Frozen Food</t>
+          <t>Meat</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>34.9</v>
+        <v>189.9</v>
       </c>
       <c r="E2" t="n">
-        <v>23.38</v>
+        <v>138.63</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2028-05-18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Green Olives 400g</t>
+          <t>Potato Chips 150g</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SKU-DEMO-DELI-001</t>
+          <t>SKU-DEMO-SNACK-001</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Deli</t>
+          <t>Snacks</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>74.90000000000001</v>
+        <v>44.9</v>
       </c>
       <c r="E3" t="n">
-        <v>52.43</v>
+        <v>28.29</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2027-08-24</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Milk Chocolate Bar 100g</t>
+          <t>Tomatoes 1kg</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SKU-DEMO-SNACK-001</t>
+          <t>SKU-DEMO-PRODUCE-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Snacks</t>
+          <t>Produce</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>39.9</v>
+        <v>24.9</v>
       </c>
       <c r="E4" t="n">
-        <v>25.14</v>
+        <v>18.67</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2028-02-07</t>
+          <t>2028-03-27</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Canned Tomatoes 400g</t>
+          <t>Toilet Paper 8-Pack</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SKU-DEMO-CANNED-001</t>
+          <t>SKU-DEMO-HOUSEHOLD-001</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Canned Goods &amp; Legumes</t>
+          <t>Household Supplies</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>24.9</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>16.18</v>
+        <v>52.14</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2028-05-06</t>
+          <t>2027-09-05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tomatoes 1kg</t>
+          <t>Ground Coffee 250g</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SKU-DEMO-PRODUCE-001</t>
+          <t>SKU-DEMO-COFFEE-001</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Produce</t>
+          <t>Coffee &amp; Tea</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24.9</v>
+        <v>129.9</v>
       </c>
       <c r="E6" t="n">
-        <v>18.67</v>
+        <v>77.94</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2027-12-10</t>
+          <t>2027-10-22</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Canned Chickpeas 400g</t>
+          <t>Paper Towels 4-Pack</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SKU-DEMO-CANNED-002</t>
+          <t>SKU-DEMO-HOUSEHOLD-002</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Canned Goods &amp; Legumes</t>
+          <t>Household Supplies</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>22.9</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>14.88</v>
+        <v>46.34</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2027-09-14</t>
+          <t>2027-08-26</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Salami 150g</t>
+          <t>Red Apples 1kg</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SKU-DEMO-DELI-002</t>
+          <t>SKU-DEMO-PRODUCE-002</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Deli</t>
+          <t>Produce</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>54.9</v>
+        <v>27.9</v>
       </c>
       <c r="E8" t="n">
-        <v>38.43</v>
+        <v>20.92</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2028-01-22</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cheddar Cheese 400g</t>
+          <t>Orange Juice 1L</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SKU-DEMO-DAIRY-001</t>
+          <t>SKU-DEMO-BEV-001</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dairy</t>
+          <t>Beverages</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>89.90000000000001</v>
+        <v>44.9</v>
       </c>
       <c r="E9" t="n">
-        <v>61.13</v>
+        <v>27.84</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2027-12-07</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ground Beef 500g</t>
+          <t>Laundry Detergent 1.5L</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SKU-DEMO-MEAT-001</t>
+          <t>SKU-DEMO-CLEAN-001</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Meat</t>
+          <t>Cleaning Supplies</t>
         </is>
       </c>
       <c r="D10" t="n">
         <v>159.9</v>
       </c>
       <c r="E10" t="n">
-        <v>116.73</v>
+        <v>91.14</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2027-10-18</t>
+          <t>2028-07-07</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bananas 1kg</t>
+          <t>Body Wash 500ml</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SKU-DEMO-PRODUCE-002</t>
+          <t>SKU-DEMO-PERSCARE-001</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Produce</t>
+          <t>Personal Care</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>29.9</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>22.42</v>
+        <v>41.2</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2028-01-11</t>
+          <t>2028-05-03</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Ground Coffee 250g</t>
+          <t>Cola 1.5L</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SKU-DEMO-COFFEE-001</t>
+          <t>SKU-DEMO-BEV-002</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Coffee &amp; Tea</t>
+          <t>Beverages</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>129.9</v>
+        <v>34.9</v>
       </c>
       <c r="E12" t="n">
-        <v>77.94</v>
+        <v>21.64</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2028-07-10</t>
+          <t>2028-05-07</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Spaghetti 500g</t>
+          <t>Bananas 1kg</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SKU-DEMO-PANTRY-001</t>
+          <t>SKU-DEMO-PRODUCE-003</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Breakfast &amp; Pantry</t>
+          <t>Produce</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>19.9</v>
+        <v>29.9</v>
       </c>
       <c r="E13" t="n">
-        <v>12.93</v>
+        <v>22.42</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2028-05-14</t>
+          <t>2028-05-18</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mixed Nuts 200g</t>
+          <t>Black Tea Box 100ct</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SKU-DEMO-SNACK-002</t>
+          <t>SKU-DEMO-COFFEE-002</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Snacks</t>
+          <t>Coffee &amp; Tea</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>99.90000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="E14" t="n">
-        <v>62.94</v>
+        <v>53.94</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2028-07-23</t>
+          <t>2028-07-28</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Potato Chips 150g</t>
+          <t>Milk Chocolate Bar 100g</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SKU-DEMO-SNACK-003</t>
+          <t>SKU-DEMO-SNACK-002</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -829,21 +829,21 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>44.9</v>
+        <v>39.9</v>
       </c>
       <c r="E15" t="n">
-        <v>28.29</v>
+        <v>25.14</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2027-09-06</t>
+          <t>2028-01-02</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Cat Food Cans 6-Pack</t>
+          <t>Cat Litter 5kg</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -857,49 +857,49 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>89.90000000000001</v>
+        <v>149.9</v>
       </c>
       <c r="E16" t="n">
-        <v>53.94</v>
+        <v>89.94</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2028-06-09</t>
+          <t>2028-03-15</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sliced Turkey Breast 200g</t>
+          <t>Shampoo 400ml</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SKU-DEMO-DELI-003</t>
+          <t>SKU-DEMO-PERSCARE-002</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Deli</t>
+          <t>Personal Care</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>64.90000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="E17" t="n">
-        <v>45.43</v>
+        <v>49.45</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2027-09-06</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Croissant</t>
+          <t>Sourdough Baguette</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -913,362 +913,362 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>22.5</v>
+        <v>18.9</v>
       </c>
       <c r="E18" t="n">
-        <v>16.2</v>
+        <v>13.61</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Whole Milk 1L</t>
+          <t>Spaghetti 500g</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SKU-DEMO-DAIRY-002</t>
+          <t>SKU-DEMO-PANTRY-001</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Dairy</t>
+          <t>Breakfast &amp; Pantry</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>45.9</v>
+        <v>19.9</v>
       </c>
       <c r="E19" t="n">
-        <v>31.21</v>
+        <v>12.93</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2028-08-15</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Greek Yogurt 500g</t>
+          <t>Trash Bags 30ct</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SKU-DEMO-DAIRY-003</t>
+          <t>SKU-DEMO-HOUSEHOLD-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Dairy</t>
+          <t>Household Supplies</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>38.5</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="E20" t="n">
-        <v>26.18</v>
+        <v>37.64</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2027-08-30</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Chicken Breast 1kg</t>
+          <t>Baby Diapers Pack</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SKU-DEMO-MEAT-002</t>
+          <t>SKU-DEMO-BABY-001</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Meat</t>
+          <t>Baby Products</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>189.9</v>
+        <v>159.9</v>
       </c>
       <c r="E21" t="n">
-        <v>138.63</v>
+        <v>95.94</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2028-07-25</t>
+          <t>2028-03-14</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Honey 450g</t>
+          <t>Whole Milk 1L</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SKU-DEMO-PANTRY-002</t>
+          <t>SKU-DEMO-DAIRY-001</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Breakfast &amp; Pantry</t>
+          <t>Dairy</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>149.9</v>
+        <v>45.9</v>
       </c>
       <c r="E22" t="n">
-        <v>97.44</v>
+        <v>31.21</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2028-01-26</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Instant Coffee 200g</t>
+          <t>White Bread Loaf</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SKU-DEMO-COFFEE-002</t>
+          <t>SKU-DEMO-BAKERY-002</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Coffee &amp; Tea</t>
+          <t>Bakery</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>149.9</v>
+        <v>15.9</v>
       </c>
       <c r="E23" t="n">
-        <v>89.94</v>
+        <v>11.45</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2028-03-27</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Cat Litter 5kg</t>
+          <t>Lamb Chops 500g</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SKU-DEMO-PET-002</t>
+          <t>SKU-DEMO-MEAT-002</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pet Supplies</t>
+          <t>Meat</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>149.9</v>
+        <v>249.9</v>
       </c>
       <c r="E24" t="n">
-        <v>89.94</v>
+        <v>182.43</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2028-03-12</t>
+          <t>2028-08-10</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Frozen Pizza</t>
+          <t>Honey 450g</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SKU-DEMO-FROZEN-002</t>
+          <t>SKU-DEMO-PANTRY-002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Frozen Food</t>
+          <t>Breakfast &amp; Pantry</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>89.90000000000001</v>
+        <v>149.9</v>
       </c>
       <c r="E25" t="n">
-        <v>60.23</v>
+        <v>97.44</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2027-09-08</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Canned Tuna 150g</t>
+          <t>Vanilla Ice Cream 1L</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SKU-DEMO-CANNED-003</t>
+          <t>SKU-DEMO-FROZEN-001</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Canned Goods &amp; Legumes</t>
+          <t>Frozen Food</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>39.9</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="E26" t="n">
-        <v>25.93</v>
+        <v>53.53</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2028-05-21</t>
+          <t>2026-09-27</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Laundry Detergent 1.5L</t>
+          <t>Toothpaste 100ml</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SKU-DEMO-CLEAN-001</t>
+          <t>SKU-DEMO-PERSCARE-003</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Cleaning Supplies</t>
+          <t>Personal Care</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>159.9</v>
+        <v>54.9</v>
       </c>
       <c r="E27" t="n">
-        <v>91.14</v>
+        <v>30.2</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2027-10-15</t>
+          <t>2028-04-22</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dry Dog Food 2kg</t>
+          <t>Cheddar Cheese 400g</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SKU-DEMO-PET-003</t>
+          <t>SKU-DEMO-DAIRY-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Pet Supplies</t>
+          <t>Dairy</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>199.9</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="E28" t="n">
-        <v>119.94</v>
+        <v>61.13</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2027-09-23</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Orange Juice 1L</t>
+          <t>Cat Food Cans 6-Pack</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SKU-DEMO-BEV-001</t>
+          <t>SKU-DEMO-PET-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Beverages</t>
+          <t>Pet Supplies</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>44.9</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="E29" t="n">
-        <v>27.84</v>
+        <v>53.94</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2028-04-17</t>
+          <t>2028-01-06</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Black Tea Box 100ct</t>
+          <t>Green Olives 400g</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SKU-DEMO-COFFEE-003</t>
+          <t>SKU-DEMO-DELI-001</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Coffee &amp; Tea</t>
+          <t>Deli</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>89.90000000000001</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="E30" t="n">
-        <v>53.94</v>
+        <v>52.43</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2027-09-03</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Sourdough Baguette</t>
+          <t>Croissant</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SKU-DEMO-BAKERY-002</t>
+          <t>SKU-DEMO-BAKERY-003</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1277,518 +1277,518 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>18.9</v>
+        <v>22.5</v>
       </c>
       <c r="E31" t="n">
-        <v>13.61</v>
+        <v>16.2</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Paper Towels 4-Pack</t>
+          <t>Greek Yogurt 500g</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SKU-DEMO-HOUSEHOLD-001</t>
+          <t>SKU-DEMO-DAIRY-003</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Household Supplies</t>
+          <t>Dairy</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>79.90000000000001</v>
+        <v>38.5</v>
       </c>
       <c r="E32" t="n">
-        <v>46.34</v>
+        <v>26.18</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2028-01-01</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Multi-Surface Cleaner 500ml</t>
+          <t>Corn Flakes 500g</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>SKU-DEMO-CLEAN-002</t>
+          <t>SKU-DEMO-PANTRY-003</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Cleaning Supplies</t>
+          <t>Breakfast &amp; Pantry</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>44.9</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="E33" t="n">
-        <v>25.59</v>
+        <v>42.19</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2028-07-29</t>
+          <t>2027-10-12</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Baby Wipes Pack</t>
+          <t>Canned Tomatoes 400g</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SKU-DEMO-BABY-001</t>
+          <t>SKU-DEMO-CANNED-001</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Baby Products</t>
+          <t>Canned Goods &amp; Legumes</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>49.9</v>
+        <v>24.9</v>
       </c>
       <c r="E34" t="n">
-        <v>29.94</v>
+        <v>16.18</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2027-12-20</t>
+          <t>2027-08-19</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Lamb Chops 500g</t>
+          <t>Mixed Nuts 200g</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SKU-DEMO-MEAT-003</t>
+          <t>SKU-DEMO-SNACK-003</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Meat</t>
+          <t>Snacks</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>249.9</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="E35" t="n">
-        <v>182.43</v>
+        <v>62.94</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2027-08-26</t>
+          <t>2027-09-20</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>White Bread Loaf</t>
+          <t>Dry Dog Food 2kg</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SKU-DEMO-BAKERY-003</t>
+          <t>SKU-DEMO-PET-003</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Bakery</t>
+          <t>Pet Supplies</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>15.9</v>
+        <v>199.9</v>
       </c>
       <c r="E36" t="n">
-        <v>11.45</v>
+        <v>119.94</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2028-02-13</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Corn Flakes 500g</t>
+          <t>Frozen Pizza</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SKU-DEMO-PANTRY-003</t>
+          <t>SKU-DEMO-FROZEN-002</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Breakfast &amp; Pantry</t>
+          <t>Frozen Food</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>64.90000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="E37" t="n">
-        <v>42.19</v>
+        <v>60.23</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2028-07-26</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Toilet Paper 8-Pack</t>
+          <t>Baby Wipes Pack</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SKU-DEMO-HOUSEHOLD-002</t>
+          <t>SKU-DEMO-BABY-002</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Household Supplies</t>
+          <t>Baby Products</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>89.90000000000001</v>
+        <v>49.9</v>
       </c>
       <c r="E38" t="n">
-        <v>52.14</v>
+        <v>29.94</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2028-01-31</t>
+          <t>2027-11-15</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Red Apples 1kg</t>
+          <t>Canned Tuna 150g</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SKU-DEMO-PRODUCE-003</t>
+          <t>SKU-DEMO-CANNED-002</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Produce</t>
+          <t>Canned Goods &amp; Legumes</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>27.9</v>
+        <v>39.9</v>
       </c>
       <c r="E39" t="n">
-        <v>20.92</v>
+        <v>25.93</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2028-07-11</t>
+          <t>2028-04-10</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Cola 1.5L</t>
+          <t>Baby Formula 800g</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SKU-DEMO-BEV-002</t>
+          <t>SKU-DEMO-BABY-003</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Beverages</t>
+          <t>Baby Products</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>34.9</v>
+        <v>349.9</v>
       </c>
       <c r="E40" t="n">
-        <v>21.64</v>
+        <v>209.94</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2027-12-05</t>
+          <t>2028-01-28</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Toothpaste 100ml</t>
+          <t>Multi-Surface Cleaner 500ml</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SKU-DEMO-PERSCARE-001</t>
+          <t>SKU-DEMO-CLEAN-002</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Personal Care</t>
+          <t>Cleaning Supplies</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>54.9</v>
+        <v>44.9</v>
       </c>
       <c r="E41" t="n">
-        <v>30.2</v>
+        <v>25.59</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2028-03-19</t>
+          <t>2028-01-14</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Baby Formula 800g</t>
+          <t>Salami 150g</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SKU-DEMO-BABY-002</t>
+          <t>SKU-DEMO-DELI-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Baby Products</t>
+          <t>Deli</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>349.9</v>
+        <v>54.9</v>
       </c>
       <c r="E42" t="n">
-        <v>209.94</v>
+        <v>38.43</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2028-02-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dish Soap 750ml</t>
+          <t>Sparkling Water 500ml</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SKU-DEMO-CLEAN-003</t>
+          <t>SKU-DEMO-BEV-003</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Cleaning Supplies</t>
+          <t>Beverages</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>49.9</v>
+        <v>12.9</v>
       </c>
       <c r="E43" t="n">
-        <v>28.44</v>
+        <v>8</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2028-03-03</t>
+          <t>2028-07-24</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Trash Bags 30ct</t>
+          <t>Frozen Peas 500g</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SKU-DEMO-HOUSEHOLD-003</t>
+          <t>SKU-DEMO-FROZEN-003</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Household Supplies</t>
+          <t>Frozen Food</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>64.90000000000001</v>
+        <v>34.9</v>
       </c>
       <c r="E44" t="n">
-        <v>37.64</v>
+        <v>23.38</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2027-09-02</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Baby Diapers Pack</t>
+          <t>Ground Beef 500g</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SKU-DEMO-BABY-003</t>
+          <t>SKU-DEMO-MEAT-003</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Baby Products</t>
+          <t>Meat</t>
         </is>
       </c>
       <c r="D45" t="n">
         <v>159.9</v>
       </c>
       <c r="E45" t="n">
-        <v>95.94</v>
+        <v>116.73</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2027-12-29</t>
+          <t>2027-09-03</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Vanilla Ice Cream 1L</t>
+          <t>Instant Coffee 200g</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SKU-DEMO-FROZEN-003</t>
+          <t>SKU-DEMO-COFFEE-003</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Frozen Food</t>
+          <t>Coffee &amp; Tea</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>79.90000000000001</v>
+        <v>149.9</v>
       </c>
       <c r="E46" t="n">
-        <v>53.53</v>
+        <v>89.94</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2027-11-03</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Shampoo 400ml</t>
+          <t>Canned Chickpeas 400g</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SKU-DEMO-PERSCARE-002</t>
+          <t>SKU-DEMO-CANNED-003</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Personal Care</t>
+          <t>Canned Goods &amp; Legumes</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>89.90000000000001</v>
+        <v>22.9</v>
       </c>
       <c r="E47" t="n">
-        <v>49.45</v>
+        <v>14.88</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2027-10-03</t>
+          <t>2028-05-15</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Sparkling Water 500ml</t>
+          <t>Dish Soap 750ml</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SKU-DEMO-BEV-003</t>
+          <t>SKU-DEMO-CLEAN-003</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Beverages</t>
+          <t>Cleaning Supplies</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>12.9</v>
+        <v>49.9</v>
       </c>
       <c r="E48" t="n">
-        <v>8</v>
+        <v>28.44</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2028-06-09</t>
+          <t>2027-12-04</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Body Wash 500ml</t>
+          <t>Sliced Turkey Breast 200g</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SKU-DEMO-PERSCARE-003</t>
+          <t>SKU-DEMO-DELI-003</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Personal Care</t>
+          <t>Deli</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>74.90000000000001</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="E49" t="n">
-        <v>41.2</v>
+        <v>45.43</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2027-11-14</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>

</xml_diff>